<commit_message>
Update app logic and generated output workbooks.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1048,7 +1048,7 @@
     <col hidden="1" width="0.727272727272727" customWidth="1" style="1" min="1" max="1"/>
     <col width="0.454545454545455" customWidth="1" style="1" min="2" max="2"/>
     <col width="5.36363636363636" customWidth="1" style="1" min="3" max="3"/>
-    <col width="38.3636363636364" customWidth="1" style="1" min="5" max="5"/>
+    <col width="52.8181818181818" customWidth="1" style="1" min="5" max="5"/>
     <col width="5.72727272727273" customWidth="1" style="1" min="6" max="6"/>
     <col width="7.18181818181818" customWidth="1" style="1" min="7" max="7"/>
     <col width="8.36363636363636" customWidth="1" style="1" min="8" max="8"/>
@@ -1101,11 +1101,6 @@
           <t>数量/Quantity</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>备注/Remarks</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="C5" s="4" t="n"/>
@@ -1138,41 +1133,45 @@
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="0" t="n"/>
-      <c r="G8" s="0" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
       <c r="I8" s="0" t="n"/>
     </row>
     <row r="9">
       <c r="C9" s="4" t="n"/>
-      <c r="E9" s="0" t="n"/>
-      <c r="F9" s="0" t="n"/>
-      <c r="G9" s="0" t="n"/>
-      <c r="H9" s="0" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
       <c r="I9" s="0" t="n"/>
     </row>
     <row r="10">
       <c r="C10" s="4" t="n"/>
-      <c r="E10" s="0" t="n"/>
-      <c r="F10" s="0" t="n"/>
-      <c r="G10" s="0" t="n"/>
-      <c r="H10" s="0" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
       <c r="I10" s="0" t="n"/>
     </row>
     <row r="11">
       <c r="C11" s="4" t="n"/>
-      <c r="E11" s="0" t="n"/>
-      <c r="F11" s="0" t="n"/>
-      <c r="G11" s="0" t="n"/>
-      <c r="H11" s="0" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
       <c r="I11" s="0" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="4" t="n"/>
-      <c r="E12" s="0" t="n"/>
-      <c r="F12" s="0" t="n"/>
-      <c r="G12" s="0" t="n"/>
-      <c r="H12" s="0" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
       <c r="I12" s="0" t="n"/>
     </row>
     <row r="13">

</xml_diff>